<commit_message>
✨ feat: add grid constraint support for assemblies
- Add GridConstraint and GridInflation data classes
- Add AssemblyGridConstraint for mapping constraints to assemblies
- Support wildcard pattern matching for assembly names
- Build grid_constraint_att elements in attributes section
- Apply x/y/z/all_grid_constraint to assembly elements
- Update Excel template with grid_constraints and assembly_constraints sheets

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/grid_template.xlsx
+++ b/grid_template.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet name="system_grid" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="grid_patches" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="grid_constraints" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="assembly_constraints" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -773,4 +775,220 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>enable_min_cell_size</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>min_cell_size</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>number_cells_control</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>max_size</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>min_number</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fin_Constraint</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>min_number</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="F2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>鳍片区域网格约束</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Base_Constraint</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>max_size</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>基座区域网格约束</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>assembly_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>x_constraint</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>y_constraint</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>z_constraint</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>all_constraint</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fin*</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fin_Constraint</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>所有 Fin 开头的装配件应用 X 方向约束</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Base_Constraint</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Base 装配件应用全方向约束</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
🐛 fix: applies_to should use x_direction for y_direction, z_direction
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/grid_template.xlsx
+++ b/grid_template.xlsx
@@ -708,7 +708,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>x_direction</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -744,7 +744,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>y</t>
+          <t>y_direction</t>
         </is>
       </c>
       <c r="C3" t="n">

</xml_diff>